<commit_message>
Update House model inputs and outputs
</commit_message>
<xml_diff>
--- a/inputs/House Model Data.xlsx
+++ b/inputs/House Model Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benyelin/Developer/house_model_python/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5880301F-56C2-3A49-8CE7-516D7DD90714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B13B7A4-45C1-214B-BACD-CB50AC4A9B56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1460" yWindow="1560" windowWidth="27640" windowHeight="16940" xr2:uid="{9CA4CF23-00BE-4A4E-B0A3-B27FE202FE9A}"/>
   </bookViews>
@@ -14447,7 +14447,7 @@
         <v>698</v>
       </c>
       <c r="T198" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
     </row>
     <row r="199" spans="1:20" x14ac:dyDescent="0.2">
@@ -14502,7 +14502,7 @@
         <v>698</v>
       </c>
       <c r="T199" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
     </row>
     <row r="200" spans="1:20" x14ac:dyDescent="0.2">

</xml_diff>